<commit_message>
added negative testcase and error screenshot
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/LoginTest.xlsx
+++ b/src/test/resources/testdata/LoginTest.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30524"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{0FB8998F-49AD-4394-A0AF-180D699B4843}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{7886DC49-3762-4D2B-A2B2-F51D5AE52495}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="18">
   <si>
     <t>testCaseName</t>
   </si>
@@ -51,16 +51,43 @@
     <t>password</t>
   </si>
   <si>
+    <t>errorMsg</t>
+  </si>
+  <si>
+    <t>tabText</t>
+  </si>
+  <si>
     <t>Positive_OrangeHRM_VerifyAdminLoginWithValidUsernameAndPassword</t>
   </si>
   <si>
     <t>Positive</t>
   </si>
   <si>
+    <t>TC01_Login1</t>
+  </si>
+  <si>
     <t>Admin</t>
   </si>
   <si>
     <t>admin123</t>
+  </si>
+  <si>
+    <t>Dashboard</t>
+  </si>
+  <si>
+    <t>Negative_OrangeHRM_VerifyLoginWithInvalidUsernameAndValidPassword_withInvalidCredentailsError</t>
+  </si>
+  <si>
+    <t>Negative</t>
+  </si>
+  <si>
+    <t>TC01_Login2</t>
+  </si>
+  <si>
+    <t>Admin12</t>
+  </si>
+  <si>
+    <t>Invalid credentials</t>
   </si>
 </sst>
 </file>
@@ -412,13 +439,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:G3"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="3" max="3" width="10.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:7">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -434,22 +461,51 @@
       <c r="E1" t="s">
         <v>4</v>
       </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
     </row>
-    <row r="2" spans="1:5">
+    <row r="2" spans="1:7">
       <c r="A2" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="B2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C2">
-        <v>152281126</v>
+        <v>8</v>
+      </c>
+      <c r="C2" t="s">
+        <v>9</v>
       </c>
       <c r="D2" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="E2" t="s">
-        <v>8</v>
+        <v>11</v>
+      </c>
+      <c r="G2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7">
+      <c r="A3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C3" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3" t="s">
+        <v>16</v>
+      </c>
+      <c r="E3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F3" t="s">
+        <v>17</v>
       </c>
     </row>
   </sheetData>

</xml_diff>